<commit_message>
Fix: Update test artifacts and bug reports for portfolio completeness
</commit_message>
<xml_diff>
--- a/manual-testing/test-design-techniques/boundary-value-analysis.xlsx
+++ b/manual-testing/test-design-techniques/boundary-value-analysis.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16965" windowHeight="5655" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16965" windowHeight="5655"/>
   </bookViews>
   <sheets>
     <sheet name="Phone BVA" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="113">
   <si>
     <t>Test ID</t>
   </si>
@@ -362,13 +362,19 @@
   </si>
   <si>
     <t>10.5</t>
+  </si>
+  <si>
+    <t>Bu tablo test tasarımı aşamasını göstermektedir. Test execution sonuçları test-cases.xlsx dosyasında takip edilmiştir.</t>
+  </si>
+  <si>
+    <t>Notes:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -381,6 +387,24 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="162"/>
@@ -548,7 +572,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
@@ -626,6 +650,8 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -906,7 +932,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="13.7109375" customWidth="1"/>
@@ -1168,6 +1194,22 @@
       <c r="F13" s="3"/>
       <c r="G13" s="4"/>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="29" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1176,7 +1218,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1401,6 +1443,20 @@
       <c r="F11" s="17"/>
       <c r="G11" s="25"/>
     </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="B14" s="30"/>
+      <c r="C14" s="30"/>
+      <c r="D14" s="30"/>
+      <c r="E14" s="30"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="29" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1408,7 +1464,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -1690,6 +1746,20 @@
       <c r="F14" s="17"/>
       <c r="G14" s="25"/>
     </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="30" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="29" t="s">
+        <v>111</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>